<commit_message>
Give coaches editable profiles and a real activity scorecard.
Coaches can be edited, deactivated, or deleted, and classes record who taught them. The unused attendance screens are removed.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/Niik_source/NiikSkate_Ticks_Manual.xlsx
+++ b/data/Niik_source/NiikSkate_Ticks_Manual.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amdocs-my.sharepoint.com/personal/rodrigs_amdocs_com/Documents/Documents/GitHub/niikskate/data/Niik_source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="138" documentId="8_{430FBCCC-350F-43FF-86AD-68FCD4FAAC39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1870544E-7B33-4712-9BC4-7027637C2A3F}"/>
+  <xr:revisionPtr revIDLastSave="147" documentId="8_{430FBCCC-350F-43FF-86AD-68FCD4FAAC39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E28AD11E-9A28-43FD-BBCE-3EF36DB4CA7D}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Skate_Manual" sheetId="1" r:id="rId1"/>
@@ -4939,7 +4939,7 @@
         <v>353</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>250</v>
+        <v>390</v>
       </c>
       <c r="G44" s="32" t="s">
         <v>387</v>
@@ -4975,7 +4975,7 @@
         <v>353</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>250</v>
+        <v>390</v>
       </c>
       <c r="G45" s="32" t="s">
         <v>387</v>
@@ -5201,7 +5201,7 @@
         <v>353</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>250</v>
+        <v>390</v>
       </c>
       <c r="G51" s="32" t="s">
         <v>387</v>
@@ -5237,7 +5237,7 @@
         <v>353</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>250</v>
+        <v>390</v>
       </c>
       <c r="G52" s="32" t="s">
         <v>387</v>
@@ -5597,7 +5597,7 @@
         <v>353</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>250</v>
+        <v>390</v>
       </c>
       <c r="G62" s="32" t="s">
         <v>387</v>
@@ -30911,7 +30911,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:T260" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="F261:G1018 C215 C169:C191 C94:C114 C136:C167 F112:F260">
+  <conditionalFormatting sqref="C94:C114 F112:F260 C136:C167 C169:C191 C215 F261:G1018">
     <cfRule type="containsText" dxfId="5" priority="35" operator="containsText" text="Linea">
       <formula>NOT(ISERROR(SEARCH(("Linea"),(C94))))</formula>
     </cfRule>
@@ -30919,7 +30919,7 @@
       <formula>NOT(ISERROR(SEARCH(("Juego"),(C94))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F261:G1018 C215 C169:C191 C94:C114 C136:C167 F112:F260">
+  <conditionalFormatting sqref="F112:F260 C94:C114 C136:C167 C169:C191 C215 F261:G1018">
     <cfRule type="containsText" dxfId="3" priority="34" operator="containsText" text="Truco">
       <formula>NOT(ISERROR(SEARCH(("Truco"),(C94))))</formula>
     </cfRule>

</xml_diff>